<commit_message>
added motorsport custom fonts
more ttf and otf fonts in fonts directory
</commit_message>
<xml_diff>
--- a/Documents/Datasources PowerTune.xlsx
+++ b/Documents/Datasources PowerTune.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qt61694\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PowerTuneDev\powertune_official_repo_clone\PowerTuneDigitalOfficial\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DF95B0A-BA19-42AA-A2C9-45FFE463151E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="11625" windowHeight="8490"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -5583,7 +5584,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -5724,7 +5725,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -5744,15 +5745,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6032,22 +6030,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P385"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:P225"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="43.7109375" customWidth="1"/>
-    <col min="3" max="4" width="24.85546875" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" customWidth="1"/>
-    <col min="7" max="7" width="14.85546875" customWidth="1"/>
-    <col min="8" max="8" width="14.5703125" customWidth="1"/>
-    <col min="9" max="9" width="15" customWidth="1"/>
-    <col min="10" max="10" width="19" customWidth="1"/>
-    <col min="11" max="12" width="21.28515625" customWidth="1"/>
-    <col min="13" max="14" width="12.7109375" customWidth="1"/>
-    <col min="15" max="15" width="16" customWidth="1"/>
+    <col min="2" max="2" width="36.140625" customWidth="1"/>
+    <col min="3" max="3" width="17.42578125" customWidth="1"/>
+    <col min="4" max="4" width="8" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="8.140625" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="9.5703125" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="7.42578125" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="7.85546875" hidden="1" customWidth="1"/>
+    <col min="10" max="11" width="7.5703125" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11" customWidth="1"/>
+    <col min="14" max="14" width="6" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="4.5703125" hidden="1" customWidth="1"/>
     <col min="16" max="16" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6102,10 +6103,10 @@
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="2" t="s">
         <v>1646</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="2" t="s">
         <v>267</v>
       </c>
       <c r="C2" s="12" t="s">
@@ -6141,11 +6142,11 @@
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+    <row r="3" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B3" s="13"/>
+      <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
@@ -6165,11 +6166,11 @@
       <c r="O3" s="2"/>
       <c r="P3" s="2"/>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+    <row r="4" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="2" t="s">
         <v>220</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -6213,11 +6214,11 @@
         <v>150</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+    <row r="5" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="2" t="s">
         <v>221</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -6261,11 +6262,11 @@
         <v>150</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
+    <row r="6" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="2" t="s">
         <v>222</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -6309,11 +6310,11 @@
         <v>150</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+    <row r="7" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="2" t="s">
         <v>238</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -6353,11 +6354,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
+    <row r="8" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>1798</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="2" t="s">
         <v>301</v>
       </c>
       <c r="C8" s="12" t="s">
@@ -6393,11 +6394,11 @@
       <c r="O8" s="2"/>
       <c r="P8" s="2"/>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A9" s="13" t="s">
+    <row r="9" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="2" t="s">
         <v>219</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -6437,11 +6438,11 @@
         <v>150</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
+    <row r="10" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="2" t="s">
         <v>218</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -6479,11 +6480,11 @@
         <v>150</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" s="13" t="s">
+    <row r="11" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>1702</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="2" t="s">
         <v>334</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -6519,11 +6520,11 @@
       <c r="O11" s="2"/>
       <c r="P11" s="2"/>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A12" s="13" t="s">
+    <row r="12" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>1701</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="2" t="s">
         <v>333</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -6559,11 +6560,11 @@
       <c r="O12" s="2"/>
       <c r="P12" s="2"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A13" s="13" t="s">
+    <row r="13" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="2" t="s">
         <v>1843</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -6601,11 +6602,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A14" s="13" t="s">
+    <row r="14" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="2" t="s">
         <v>1845</v>
       </c>
       <c r="C14" s="2"/>
@@ -6641,11 +6642,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A15" s="13" t="s">
+    <row r="15" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B15" s="13"/>
+      <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="5" t="s">
@@ -6679,11 +6680,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A16" s="13" t="s">
+    <row r="16" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B16" s="13"/>
+      <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="5" t="s">
@@ -6718,10 +6719,10 @@
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="2" t="s">
         <v>1703</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="2" t="s">
         <v>335</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -6757,11 +6758,11 @@
       <c r="O17" s="2"/>
       <c r="P17" s="2"/>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A18" s="13" t="s">
+    <row r="18" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="B18" s="13"/>
+      <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="5" t="s">
@@ -6796,10 +6797,10 @@
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A19" s="13" t="s">
+      <c r="A19" s="2" t="s">
         <v>1689</v>
       </c>
-      <c r="B19" s="13" t="s">
+      <c r="B19" s="2" t="s">
         <v>320</v>
       </c>
       <c r="C19" s="12"/>
@@ -6834,10 +6835,10 @@
       <c r="P19" s="2"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="13" t="s">
+      <c r="B20" s="2" t="s">
         <v>234</v>
       </c>
       <c r="C20" s="2" t="s">
@@ -6878,10 +6879,10 @@
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A21" s="13" t="s">
+      <c r="A21" s="2" t="s">
         <v>1710</v>
       </c>
-      <c r="B21" s="13" t="s">
+      <c r="B21" s="2" t="s">
         <v>342</v>
       </c>
       <c r="C21" s="2" t="s">
@@ -6918,10 +6919,10 @@
       <c r="P21" s="2"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A22" s="13" t="s">
+      <c r="A22" s="2" t="s">
         <v>1735</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="2" t="s">
         <v>294</v>
       </c>
       <c r="C22" s="12" t="s">
@@ -6957,11 +6958,11 @@
       <c r="O22" s="2"/>
       <c r="P22" s="2"/>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A23" s="13" t="s">
+    <row r="23" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B23" s="13" t="s">
+      <c r="B23" s="2" t="s">
         <v>239</v>
       </c>
       <c r="C23" s="2" t="s">
@@ -6999,11 +7000,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A24" s="13" t="s">
+    <row r="24" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B24" s="13" t="s">
+      <c r="B24" s="2" t="s">
         <v>166</v>
       </c>
       <c r="C24" s="2" t="s">
@@ -7039,11 +7040,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A25" s="13" t="s">
+    <row r="25" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B25" s="13"/>
+      <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
       <c r="E25" s="3" t="s">
@@ -7077,11 +7078,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A26" s="13" t="s">
+    <row r="26" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B26" s="13"/>
+      <c r="B26" s="2"/>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
       <c r="E26" s="3" t="s">
@@ -7116,10 +7117,10 @@
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A27" s="13" t="s">
+      <c r="A27" s="2" t="s">
         <v>1699</v>
       </c>
-      <c r="B27" s="13" t="s">
+      <c r="B27" s="2" t="s">
         <v>331</v>
       </c>
       <c r="C27" s="2" t="s">
@@ -7156,10 +7157,10 @@
       <c r="P27" s="2"/>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A28" s="13" t="s">
+      <c r="A28" s="2" t="s">
         <v>1657</v>
       </c>
-      <c r="B28" s="13" t="s">
+      <c r="B28" s="2" t="s">
         <v>282</v>
       </c>
       <c r="C28" s="12"/>
@@ -7194,10 +7195,10 @@
       <c r="P28" s="2"/>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A29" s="13" t="s">
+      <c r="A29" s="2" t="s">
         <v>1700</v>
       </c>
-      <c r="B29" s="13" t="s">
+      <c r="B29" s="2" t="s">
         <v>332</v>
       </c>
       <c r="C29" s="2" t="s">
@@ -7233,11 +7234,11 @@
       <c r="O29" s="2"/>
       <c r="P29" s="2"/>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A30" s="13" t="s">
+    <row r="30" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="B30" s="13" t="s">
+      <c r="B30" s="2" t="s">
         <v>227</v>
       </c>
       <c r="C30" s="2"/>
@@ -7276,10 +7277,10 @@
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A31" s="13" t="s">
+      <c r="A31" s="2" t="s">
         <v>1643</v>
       </c>
-      <c r="B31" s="13" t="s">
+      <c r="B31" s="2" t="s">
         <v>265</v>
       </c>
       <c r="C31" s="12" t="s">
@@ -7316,10 +7317,10 @@
       <c r="P31" s="2"/>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A32" s="13" t="s">
+      <c r="A32" s="2" t="s">
         <v>1696</v>
       </c>
-      <c r="B32" s="13" t="s">
+      <c r="B32" s="2" t="s">
         <v>329</v>
       </c>
       <c r="C32" s="2" t="s">
@@ -7356,10 +7357,10 @@
       <c r="P32" s="2"/>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A33" s="13" t="s">
+      <c r="A33" s="2" t="s">
         <v>1686</v>
       </c>
-      <c r="B33" s="13" t="s">
+      <c r="B33" s="2" t="s">
         <v>316</v>
       </c>
       <c r="C33" s="12" t="s">
@@ -7396,10 +7397,10 @@
       <c r="P33" s="2"/>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A34" s="13" t="s">
+      <c r="A34" s="2" t="s">
         <v>1690</v>
       </c>
-      <c r="B34" s="13" t="s">
+      <c r="B34" s="2" t="s">
         <v>321</v>
       </c>
       <c r="C34" s="12"/>
@@ -7423,21 +7424,21 @@
         <v>161</v>
       </c>
       <c r="K34" s="12"/>
-      <c r="L34" s="16" t="s">
+      <c r="L34" s="14" t="s">
         <v>1808</v>
       </c>
-      <c r="M34" s="16" t="s">
+      <c r="M34" s="14" t="s">
         <v>150</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
       <c r="P34" s="2"/>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A35" s="13" t="s">
+    <row r="35" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B35" s="13"/>
+      <c r="B35" s="2"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
       <c r="E35" s="3" t="s">
@@ -7472,10 +7473,10 @@
       </c>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A36" s="13" t="s">
+      <c r="A36" s="2" t="s">
         <v>1659</v>
       </c>
-      <c r="B36" s="13" t="s">
+      <c r="B36" s="2" t="s">
         <v>302</v>
       </c>
       <c r="C36" s="12" t="s">
@@ -7512,10 +7513,10 @@
       <c r="P36" s="2"/>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A37" s="13" t="s">
+      <c r="A37" s="2" t="s">
         <v>1669</v>
       </c>
-      <c r="B37" s="13" t="s">
+      <c r="B37" s="2" t="s">
         <v>303</v>
       </c>
       <c r="C37" s="12" t="s">
@@ -7552,10 +7553,10 @@
       <c r="P37" s="2"/>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A38" s="13" t="s">
+      <c r="A38" s="2" t="s">
         <v>1670</v>
       </c>
-      <c r="B38" s="13" t="s">
+      <c r="B38" s="2" t="s">
         <v>304</v>
       </c>
       <c r="C38" s="12" t="s">
@@ -7592,10 +7593,10 @@
       <c r="P38" s="2"/>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A39" s="13" t="s">
+      <c r="A39" s="2" t="s">
         <v>1671</v>
       </c>
-      <c r="B39" s="13" t="s">
+      <c r="B39" s="2" t="s">
         <v>305</v>
       </c>
       <c r="C39" s="12" t="s">
@@ -7632,10 +7633,10 @@
       <c r="P39" s="2"/>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A40" s="13" t="s">
+      <c r="A40" s="2" t="s">
         <v>1672</v>
       </c>
-      <c r="B40" s="13" t="s">
+      <c r="B40" s="2" t="s">
         <v>306</v>
       </c>
       <c r="C40" s="12" t="s">
@@ -7672,10 +7673,10 @@
       <c r="P40" s="2"/>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A41" s="13" t="s">
+      <c r="A41" s="2" t="s">
         <v>1673</v>
       </c>
-      <c r="B41" s="13" t="s">
+      <c r="B41" s="2" t="s">
         <v>307</v>
       </c>
       <c r="C41" s="12" t="s">
@@ -7712,10 +7713,10 @@
       <c r="P41" s="2"/>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A42" s="13" t="s">
+      <c r="A42" s="2" t="s">
         <v>1674</v>
       </c>
-      <c r="B42" s="13" t="s">
+      <c r="B42" s="2" t="s">
         <v>308</v>
       </c>
       <c r="C42" s="12" t="s">
@@ -7752,10 +7753,10 @@
       <c r="P42" s="2"/>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A43" s="13" t="s">
+      <c r="A43" s="2" t="s">
         <v>1675</v>
       </c>
-      <c r="B43" s="13" t="s">
+      <c r="B43" s="2" t="s">
         <v>309</v>
       </c>
       <c r="C43" s="12" t="s">
@@ -7792,10 +7793,10 @@
       <c r="P43" s="2"/>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A44" s="13" t="s">
+      <c r="A44" s="2" t="s">
         <v>1676</v>
       </c>
-      <c r="B44" s="13" t="s">
+      <c r="B44" s="2" t="s">
         <v>310</v>
       </c>
       <c r="C44" s="12" t="s">
@@ -7832,10 +7833,10 @@
       <c r="P44" s="2"/>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A45" s="13" t="s">
+      <c r="A45" s="2" t="s">
         <v>1677</v>
       </c>
-      <c r="B45" s="13" t="s">
+      <c r="B45" s="2" t="s">
         <v>311</v>
       </c>
       <c r="C45" s="12" t="s">
@@ -7872,10 +7873,10 @@
       <c r="P45" s="2"/>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A46" s="13" t="s">
+      <c r="A46" s="2" t="s">
         <v>1678</v>
       </c>
-      <c r="B46" s="13" t="s">
+      <c r="B46" s="2" t="s">
         <v>312</v>
       </c>
       <c r="C46" s="12" t="s">
@@ -7912,10 +7913,10 @@
       <c r="P46" s="2"/>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A47" s="13" t="s">
+      <c r="A47" s="2" t="s">
         <v>1679</v>
       </c>
-      <c r="B47" s="13" t="s">
+      <c r="B47" s="2" t="s">
         <v>313</v>
       </c>
       <c r="C47" s="12" t="s">
@@ -7951,11 +7952,11 @@
       <c r="O47" s="2"/>
       <c r="P47" s="2"/>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A48" s="13" t="s">
+    <row r="48" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B48" s="13" t="s">
+      <c r="B48" s="2" t="s">
         <v>153</v>
       </c>
       <c r="C48" s="2" t="s">
@@ -7994,10 +7995,10 @@
       </c>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A49" s="13" t="s">
+      <c r="A49" s="2" t="s">
         <v>1665</v>
       </c>
-      <c r="B49" s="13" t="s">
+      <c r="B49" s="2" t="s">
         <v>1730</v>
       </c>
       <c r="C49" s="12" t="s">
@@ -8034,10 +8035,10 @@
       <c r="P49" s="2"/>
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A50" s="13" t="s">
+      <c r="A50" s="2" t="s">
         <v>1666</v>
       </c>
-      <c r="B50" s="13" t="s">
+      <c r="B50" s="2" t="s">
         <v>1729</v>
       </c>
       <c r="C50" s="12" t="s">
@@ -8073,11 +8074,11 @@
       <c r="O50" s="2"/>
       <c r="P50" s="2"/>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A51" s="13" t="s">
+    <row r="51" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B51" s="13" t="s">
+      <c r="B51" s="2" t="s">
         <v>170</v>
       </c>
       <c r="C51" s="2" t="s">
@@ -8117,11 +8118,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A52" s="13" t="s">
+    <row r="52" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B52" s="13" t="s">
+      <c r="B52" s="2" t="s">
         <v>171</v>
       </c>
       <c r="C52" s="2" t="s">
@@ -8161,11 +8162,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A53" s="13" t="s">
+    <row r="53" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B53" s="13" t="s">
+      <c r="B53" s="2" t="s">
         <v>172</v>
       </c>
       <c r="C53" s="2" t="s">
@@ -8205,11 +8206,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A54" s="13" t="s">
+    <row r="54" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B54" s="13" t="s">
+      <c r="B54" s="2" t="s">
         <v>173</v>
       </c>
       <c r="C54" s="2" t="s">
@@ -8249,11 +8250,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A55" s="13" t="s">
+    <row r="55" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B55" s="13" t="s">
+      <c r="B55" s="2" t="s">
         <v>174</v>
       </c>
       <c r="C55" s="2" t="s">
@@ -8293,11 +8294,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A56" s="13" t="s">
+    <row r="56" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B56" s="13" t="s">
+      <c r="B56" s="2" t="s">
         <v>175</v>
       </c>
       <c r="C56" s="2" t="s">
@@ -8337,11 +8338,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A57" s="13" t="s">
+    <row r="57" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B57" s="13" t="s">
+      <c r="B57" s="2" t="s">
         <v>176</v>
       </c>
       <c r="C57" s="2" t="s">
@@ -8381,11 +8382,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A58" s="13" t="s">
+    <row r="58" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B58" s="13" t="s">
+      <c r="B58" s="2" t="s">
         <v>177</v>
       </c>
       <c r="C58" s="2" t="s">
@@ -8425,11 +8426,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A59" s="13" t="s">
+    <row r="59" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B59" s="13" t="s">
+      <c r="B59" s="2" t="s">
         <v>178</v>
       </c>
       <c r="C59" s="2" t="s">
@@ -8469,11 +8470,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A60" s="13" t="s">
+    <row r="60" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B60" s="13" t="s">
+      <c r="B60" s="2" t="s">
         <v>179</v>
       </c>
       <c r="C60" s="2" t="s">
@@ -8513,11 +8514,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A61" s="13" t="s">
+    <row r="61" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B61" s="13" t="s">
+      <c r="B61" s="2" t="s">
         <v>180</v>
       </c>
       <c r="C61" s="2" t="s">
@@ -8557,11 +8558,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A62" s="13" t="s">
+    <row r="62" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B62" s="13" t="s">
+      <c r="B62" s="2" t="s">
         <v>181</v>
       </c>
       <c r="C62" s="2" t="s">
@@ -8601,11 +8602,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A63" s="13" t="s">
+    <row r="63" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B63" s="13" t="s">
+      <c r="B63" s="2" t="s">
         <v>182</v>
       </c>
       <c r="C63" s="2" t="s">
@@ -8645,11 +8646,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A64" s="13" t="s">
+    <row r="64" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B64" s="13" t="s">
+      <c r="B64" s="2" t="s">
         <v>183</v>
       </c>
       <c r="C64" s="2" t="s">
@@ -8689,11 +8690,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A65" s="13" t="s">
+    <row r="65" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B65" s="13" t="s">
+      <c r="B65" s="2" t="s">
         <v>184</v>
       </c>
       <c r="C65" s="2" t="s">
@@ -8733,11 +8734,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A66" s="13" t="s">
+    <row r="66" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B66" s="13" t="s">
+      <c r="B66" s="2" t="s">
         <v>185</v>
       </c>
       <c r="C66" s="2" t="s">
@@ -8777,11 +8778,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A67" s="13" t="s">
+    <row r="67" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B67" s="13" t="s">
+      <c r="B67" s="2" t="s">
         <v>242</v>
       </c>
       <c r="C67" s="2" t="s">
@@ -8821,11 +8822,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A68" s="13" t="s">
+    <row r="68" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B68" s="13" t="s">
+      <c r="B68" s="2" t="s">
         <v>243</v>
       </c>
       <c r="C68" s="2" t="s">
@@ -8865,11 +8866,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A69" s="13" t="s">
+    <row r="69" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B69" s="13" t="s">
+      <c r="B69" s="2" t="s">
         <v>244</v>
       </c>
       <c r="C69" s="2" t="s">
@@ -8909,11 +8910,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A70" s="13" t="s">
+    <row r="70" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B70" s="13" t="s">
+      <c r="B70" s="2" t="s">
         <v>245</v>
       </c>
       <c r="C70" s="2" t="s">
@@ -8953,11 +8954,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A71" s="13" t="s">
+    <row r="71" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B71" s="13" t="s">
+      <c r="B71" s="2" t="s">
         <v>246</v>
       </c>
       <c r="C71" s="2" t="s">
@@ -8997,11 +8998,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A72" s="13" t="s">
+    <row r="72" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B72" s="13" t="s">
+      <c r="B72" s="2" t="s">
         <v>247</v>
       </c>
       <c r="C72" s="2" t="s">
@@ -9041,11 +9042,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A73" s="13" t="s">
+    <row r="73" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B73" s="13" t="s">
+      <c r="B73" s="2" t="s">
         <v>248</v>
       </c>
       <c r="C73" s="2" t="s">
@@ -9085,11 +9086,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A74" s="13" t="s">
+    <row r="74" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="B74" s="13" t="s">
+      <c r="B74" s="2" t="s">
         <v>249</v>
       </c>
       <c r="C74" s="2" t="s">
@@ -9129,11 +9130,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A75" s="13" t="s">
+    <row r="75" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B75" s="13" t="s">
+      <c r="B75" s="2" t="s">
         <v>250</v>
       </c>
       <c r="C75" s="2" t="s">
@@ -9173,11 +9174,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A76" s="13" t="s">
+    <row r="76" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B76" s="13" t="s">
+      <c r="B76" s="2" t="s">
         <v>251</v>
       </c>
       <c r="C76" s="2" t="s">
@@ -9217,11 +9218,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A77" s="13" t="s">
+    <row r="77" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B77" s="13" t="s">
+      <c r="B77" s="2" t="s">
         <v>252</v>
       </c>
       <c r="C77" s="2" t="s">
@@ -9261,11 +9262,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A78" s="13" t="s">
+    <row r="78" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B78" s="13" t="s">
+      <c r="B78" s="2" t="s">
         <v>253</v>
       </c>
       <c r="C78" s="2" t="s">
@@ -9305,11 +9306,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A79" s="13" t="s">
+    <row r="79" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B79" s="13" t="s">
+      <c r="B79" s="2" t="s">
         <v>254</v>
       </c>
       <c r="C79" s="2" t="s">
@@ -9349,11 +9350,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A80" s="13" t="s">
+    <row r="80" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B80" s="13" t="s">
+      <c r="B80" s="2" t="s">
         <v>255</v>
       </c>
       <c r="C80" s="2" t="s">
@@ -9393,11 +9394,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A81" s="13" t="s">
+    <row r="81" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B81" s="13" t="s">
+      <c r="B81" s="2" t="s">
         <v>256</v>
       </c>
       <c r="C81" s="2" t="s">
@@ -9437,11 +9438,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A82" s="13" t="s">
+    <row r="82" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B82" s="13" t="s">
+      <c r="B82" s="2" t="s">
         <v>257</v>
       </c>
       <c r="C82" s="2" t="s">
@@ -9482,10 +9483,10 @@
       </c>
     </row>
     <row r="83" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A83" s="13" t="s">
+      <c r="A83" s="2" t="s">
         <v>1705</v>
       </c>
-      <c r="B83" s="13" t="s">
+      <c r="B83" s="2" t="s">
         <v>337</v>
       </c>
       <c r="C83" s="2" t="s">
@@ -9511,21 +9512,21 @@
         <v>161</v>
       </c>
       <c r="K83" s="12"/>
-      <c r="L83" s="15" t="s">
+      <c r="L83" s="13" t="s">
         <v>1822</v>
       </c>
-      <c r="M83" s="15" t="s">
+      <c r="M83" s="13" t="s">
         <v>150</v>
       </c>
       <c r="N83" s="2"/>
       <c r="O83" s="2"/>
       <c r="P83" s="2"/>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A84" s="13" t="s">
+    <row r="84" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A84" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B84" s="13" t="s">
+      <c r="B84" s="2" t="s">
         <v>240</v>
       </c>
       <c r="C84" s="2" t="s">
@@ -9564,10 +9565,10 @@
       </c>
     </row>
     <row r="85" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A85" s="13" t="s">
+      <c r="A85" s="2" t="s">
         <v>1656</v>
       </c>
-      <c r="B85" s="13" t="s">
+      <c r="B85" s="2" t="s">
         <v>319</v>
       </c>
       <c r="C85" s="12"/>
@@ -9591,10 +9592,10 @@
         <v>161</v>
       </c>
       <c r="K85" s="12"/>
-      <c r="L85" s="16" t="s">
+      <c r="L85" s="14" t="s">
         <v>1806</v>
       </c>
-      <c r="M85" s="16" t="s">
+      <c r="M85" s="14" t="s">
         <v>150</v>
       </c>
       <c r="N85" s="2"/>
@@ -9602,10 +9603,10 @@
       <c r="P85" s="2"/>
     </row>
     <row r="86" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A86" s="13" t="s">
+      <c r="A86" s="2" t="s">
         <v>1687</v>
       </c>
-      <c r="B86" s="13" t="s">
+      <c r="B86" s="2" t="s">
         <v>317</v>
       </c>
       <c r="C86" s="12" t="s">
@@ -9642,10 +9643,10 @@
       <c r="P86" s="2"/>
     </row>
     <row r="87" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A87" s="13" t="s">
+      <c r="A87" s="2" t="s">
         <v>1688</v>
       </c>
-      <c r="B87" s="13" t="s">
+      <c r="B87" s="2" t="s">
         <v>318</v>
       </c>
       <c r="C87" s="12"/>
@@ -9680,10 +9681,10 @@
       <c r="P87" s="2"/>
     </row>
     <row r="88" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A88" s="13" t="s">
+      <c r="A88" s="2" t="s">
         <v>1733</v>
       </c>
-      <c r="B88" s="13" t="s">
+      <c r="B88" s="2" t="s">
         <v>289</v>
       </c>
       <c r="C88" s="12" t="s">
@@ -9720,10 +9721,10 @@
       <c r="P88" s="2"/>
     </row>
     <row r="89" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A89" s="13" t="s">
+      <c r="A89" s="2" t="s">
         <v>1682</v>
       </c>
-      <c r="B89" s="13" t="s">
+      <c r="B89" s="2" t="s">
         <v>297</v>
       </c>
       <c r="C89" s="12" t="s">
@@ -9760,10 +9761,10 @@
       <c r="P89" s="2"/>
     </row>
     <row r="90" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A90" s="13" t="s">
+      <c r="A90" s="2" t="s">
         <v>1684</v>
       </c>
-      <c r="B90" s="13" t="s">
+      <c r="B90" s="2" t="s">
         <v>299</v>
       </c>
       <c r="C90" s="12" t="s">
@@ -9800,10 +9801,10 @@
       <c r="P90" s="2"/>
     </row>
     <row r="91" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A91" s="13" t="s">
+      <c r="A91" s="2" t="s">
         <v>1683</v>
       </c>
-      <c r="B91" s="13" t="s">
+      <c r="B91" s="2" t="s">
         <v>298</v>
       </c>
       <c r="C91" s="12" t="s">
@@ -9840,10 +9841,10 @@
       <c r="P91" s="2"/>
     </row>
     <row r="92" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A92" s="13" t="s">
+      <c r="A92" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B92" s="13" t="s">
+      <c r="B92" s="2" t="s">
         <v>228</v>
       </c>
       <c r="C92" s="2" t="s">
@@ -9884,10 +9885,10 @@
       </c>
     </row>
     <row r="93" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A93" s="13" t="s">
+      <c r="A93" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B93" s="13" t="s">
+      <c r="B93" s="2" t="s">
         <v>145</v>
       </c>
       <c r="C93" s="2" t="s">
@@ -9928,10 +9929,10 @@
       </c>
     </row>
     <row r="94" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A94" s="13" t="s">
+      <c r="A94" s="2" t="s">
         <v>1693</v>
       </c>
-      <c r="B94" s="13" t="s">
+      <c r="B94" s="2" t="s">
         <v>324</v>
       </c>
       <c r="C94" s="12" t="s">
@@ -9968,10 +9969,10 @@
       <c r="P94" s="2"/>
     </row>
     <row r="95" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A95" s="13" t="s">
+      <c r="A95" s="2" t="s">
         <v>1694</v>
       </c>
-      <c r="B95" s="13" t="s">
+      <c r="B95" s="2" t="s">
         <v>325</v>
       </c>
       <c r="C95" s="12" t="s">
@@ -10008,10 +10009,10 @@
       <c r="P95" s="2"/>
     </row>
     <row r="96" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A96" s="13" t="s">
+      <c r="A96" s="2" t="s">
         <v>1691</v>
       </c>
-      <c r="B96" s="13" t="s">
+      <c r="B96" s="2" t="s">
         <v>322</v>
       </c>
       <c r="C96" s="12" t="s">
@@ -10048,10 +10049,10 @@
       <c r="P96" s="2"/>
     </row>
     <row r="97" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A97" s="13" t="s">
+      <c r="A97" s="2" t="s">
         <v>1692</v>
       </c>
-      <c r="B97" s="13" t="s">
+      <c r="B97" s="2" t="s">
         <v>323</v>
       </c>
       <c r="C97" s="12" t="s">
@@ -10088,10 +10089,10 @@
       <c r="P97" s="2"/>
     </row>
     <row r="98" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A98" s="13" t="s">
+      <c r="A98" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="B98" s="13" t="s">
+      <c r="B98" s="2" t="s">
         <v>1721</v>
       </c>
       <c r="C98" s="2" t="s">
@@ -10132,10 +10133,10 @@
       </c>
     </row>
     <row r="99" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A99" s="13" t="s">
+      <c r="A99" s="2" t="s">
         <v>1697</v>
       </c>
-      <c r="B99" s="13" t="s">
+      <c r="B99" s="2" t="s">
         <v>328</v>
       </c>
       <c r="C99" s="2" t="s">
@@ -10161,21 +10162,21 @@
         <v>161</v>
       </c>
       <c r="K99" s="12"/>
-      <c r="L99" s="15" t="s">
+      <c r="L99" s="13" t="s">
         <v>1815</v>
       </c>
-      <c r="M99" s="15" t="s">
+      <c r="M99" s="13" t="s">
         <v>150</v>
       </c>
       <c r="N99" s="2"/>
       <c r="O99" s="2"/>
       <c r="P99" s="2"/>
     </row>
-    <row r="100" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A100" s="13" t="s">
+    <row r="100" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A100" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B100" s="13" t="s">
+      <c r="B100" s="2" t="s">
         <v>258</v>
       </c>
       <c r="C100" s="2" t="s">
@@ -10200,7 +10201,7 @@
       <c r="J100" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="K100" s="16" t="s">
+      <c r="K100" s="14" t="s">
         <v>150</v>
       </c>
       <c r="L100" s="5" t="s">
@@ -10215,11 +10216,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="101" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A101" s="13" t="s">
+    <row r="101" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A101" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B101" s="13" t="s">
+      <c r="B101" s="2" t="s">
         <v>259</v>
       </c>
       <c r="C101" s="2"/>
@@ -10242,7 +10243,7 @@
       <c r="J101" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="K101" s="16" t="s">
+      <c r="K101" s="14" t="s">
         <v>150</v>
       </c>
       <c r="L101" s="5" t="s">
@@ -10257,11 +10258,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="102" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A102" s="13" t="s">
+    <row r="102" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B102" s="13" t="s">
+      <c r="B102" s="2" t="s">
         <v>260</v>
       </c>
       <c r="C102" s="2"/>
@@ -10284,7 +10285,7 @@
       <c r="J102" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="K102" s="16" t="s">
+      <c r="K102" s="14" t="s">
         <v>150</v>
       </c>
       <c r="L102" s="5" t="s">
@@ -10299,11 +10300,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="103" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A103" s="13" t="s">
+    <row r="103" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A103" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B103" s="13" t="s">
+      <c r="B103" s="2" t="s">
         <v>261</v>
       </c>
       <c r="C103" s="2"/>
@@ -10326,7 +10327,7 @@
       <c r="J103" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="K103" s="16" t="s">
+      <c r="K103" s="14" t="s">
         <v>150</v>
       </c>
       <c r="L103" s="5" t="s">
@@ -10341,11 +10342,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="104" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A104" s="13" t="s">
+    <row r="104" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A104" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="B104" s="13" t="s">
+      <c r="B104" s="2" t="s">
         <v>262</v>
       </c>
       <c r="C104" s="2"/>
@@ -10368,7 +10369,7 @@
       <c r="J104" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="K104" s="16" t="s">
+      <c r="K104" s="14" t="s">
         <v>150</v>
       </c>
       <c r="L104" s="5" t="s">
@@ -10383,11 +10384,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="105" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A105" s="13" t="s">
+    <row r="105" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A105" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B105" s="13" t="s">
+      <c r="B105" s="2" t="s">
         <v>263</v>
       </c>
       <c r="C105" s="2" t="s">
@@ -10412,7 +10413,7 @@
       <c r="J105" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="K105" s="16" t="s">
+      <c r="K105" s="14" t="s">
         <v>150</v>
       </c>
       <c r="L105" s="5" t="s">
@@ -10427,11 +10428,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="106" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A106" s="13" t="s">
+    <row r="106" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A106" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="B106" s="13" t="s">
+      <c r="B106" s="2" t="s">
         <v>224</v>
       </c>
       <c r="C106" s="2"/>
@@ -10469,11 +10470,11 @@
         <v>150</v>
       </c>
     </row>
-    <row r="107" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A107" s="13" t="s">
+    <row r="107" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A107" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="B107" s="13" t="s">
+      <c r="B107" s="2" t="s">
         <v>225</v>
       </c>
       <c r="C107" s="2"/>
@@ -10511,11 +10512,11 @@
         <v>150</v>
       </c>
     </row>
-    <row r="108" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A108" s="13" t="s">
+    <row r="108" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A108" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B108" s="13" t="s">
+      <c r="B108" s="2" t="s">
         <v>226</v>
       </c>
       <c r="C108" s="2"/>
@@ -10554,10 +10555,10 @@
       </c>
     </row>
     <row r="109" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A109" s="13" t="s">
+      <c r="A109" s="2" t="s">
         <v>1715</v>
       </c>
-      <c r="B109" s="13" t="s">
+      <c r="B109" s="2" t="s">
         <v>347</v>
       </c>
       <c r="C109" s="2" t="s">
@@ -10583,10 +10584,10 @@
         <v>161</v>
       </c>
       <c r="K109" s="12"/>
-      <c r="L109" s="15" t="s">
+      <c r="L109" s="13" t="s">
         <v>1831</v>
       </c>
-      <c r="M109" s="15" t="s">
+      <c r="M109" s="13" t="s">
         <v>150</v>
       </c>
       <c r="N109" s="2"/>
@@ -10594,10 +10595,10 @@
       <c r="P109" s="2"/>
     </row>
     <row r="110" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A110" s="13" t="s">
+      <c r="A110" s="2" t="s">
         <v>1714</v>
       </c>
-      <c r="B110" s="13" t="s">
+      <c r="B110" s="2" t="s">
         <v>346</v>
       </c>
       <c r="C110" s="2" t="s">
@@ -10623,10 +10624,10 @@
         <v>161</v>
       </c>
       <c r="K110" s="12"/>
-      <c r="L110" s="15" t="s">
+      <c r="L110" s="13" t="s">
         <v>1830</v>
       </c>
-      <c r="M110" s="15" t="s">
+      <c r="M110" s="13" t="s">
         <v>150</v>
       </c>
       <c r="N110" s="2"/>
@@ -10634,10 +10635,10 @@
       <c r="P110" s="2"/>
     </row>
     <row r="111" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A111" s="13" t="s">
+      <c r="A111" s="2" t="s">
         <v>1655</v>
       </c>
-      <c r="B111" s="13" t="s">
+      <c r="B111" s="2" t="s">
         <v>276</v>
       </c>
       <c r="C111" s="12"/>
@@ -10671,11 +10672,11 @@
       <c r="O111" s="2"/>
       <c r="P111" s="2"/>
     </row>
-    <row r="112" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A112" s="13" t="s">
+    <row r="112" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A112" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B112" s="13"/>
+      <c r="B112" s="2"/>
       <c r="C112" s="2"/>
       <c r="D112" s="2"/>
       <c r="E112" s="5" t="s">
@@ -10709,11 +10710,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="113" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A113" s="13" t="s">
+    <row r="113" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A113" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B113" s="13"/>
+      <c r="B113" s="2"/>
       <c r="C113" s="2"/>
       <c r="D113" s="2"/>
       <c r="E113" s="5" t="s">
@@ -10747,11 +10748,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="114" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A114" s="13" t="s">
+    <row r="114" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A114" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B114" s="13"/>
+      <c r="B114" s="2"/>
       <c r="C114" s="2"/>
       <c r="D114" s="2"/>
       <c r="E114" s="3" t="s">
@@ -10785,11 +10786,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="115" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A115" s="13" t="s">
+    <row r="115" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A115" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B115" s="13"/>
+      <c r="B115" s="2"/>
       <c r="C115" s="2"/>
       <c r="D115" s="2"/>
       <c r="E115" s="5" t="s">
@@ -10823,11 +10824,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="116" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A116" s="13" t="s">
+    <row r="116" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A116" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B116" s="13"/>
+      <c r="B116" s="2"/>
       <c r="C116" s="2"/>
       <c r="D116" s="2"/>
       <c r="E116" s="5" t="s">
@@ -10861,11 +10862,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="117" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A117" s="13" t="s">
+    <row r="117" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A117" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="B117" s="13"/>
+      <c r="B117" s="2"/>
       <c r="C117" s="2"/>
       <c r="D117" s="2"/>
       <c r="E117" s="5" t="s">
@@ -10900,10 +10901,10 @@
       </c>
     </row>
     <row r="118" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A118" s="13" t="s">
+      <c r="A118" s="2" t="s">
         <v>1667</v>
       </c>
-      <c r="B118" s="13" t="s">
+      <c r="B118" s="2" t="s">
         <v>292</v>
       </c>
       <c r="C118" s="12" t="s">
@@ -10939,11 +10940,11 @@
       <c r="O118" s="2"/>
       <c r="P118" s="2"/>
     </row>
-    <row r="119" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A119" s="13" t="s">
+    <row r="119" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A119" s="2" t="s">
         <v>1668</v>
       </c>
-      <c r="B119" s="13" t="s">
+      <c r="B119" s="2" t="s">
         <v>293</v>
       </c>
       <c r="C119" s="12" t="s">
@@ -10981,11 +10982,11 @@
       <c r="O119" s="2"/>
       <c r="P119" s="2"/>
     </row>
-    <row r="120" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A120" s="13" t="s">
+    <row r="120" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A120" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B120" s="13"/>
+      <c r="B120" s="2"/>
       <c r="C120" s="2"/>
       <c r="D120" s="2"/>
       <c r="E120" s="3" t="s">
@@ -11019,11 +11020,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="121" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A121" s="13" t="s">
+    <row r="121" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A121" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B121" s="13"/>
+      <c r="B121" s="2"/>
       <c r="C121" s="2"/>
       <c r="D121" s="2"/>
       <c r="E121" s="5" t="s">
@@ -11057,11 +11058,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="122" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A122" s="13" t="s">
+    <row r="122" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A122" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="B122" s="13"/>
+      <c r="B122" s="2"/>
       <c r="C122" s="2"/>
       <c r="D122" s="2"/>
       <c r="E122" s="5" t="s">
@@ -11095,11 +11096,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="123" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A123" s="13" t="s">
+    <row r="123" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A123" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B123" s="13"/>
+      <c r="B123" s="2"/>
       <c r="C123" s="2"/>
       <c r="D123" s="2"/>
       <c r="E123" s="5" t="s">
@@ -11133,11 +11134,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="124" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A124" s="13" t="s">
+    <row r="124" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A124" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="B124" s="13"/>
+      <c r="B124" s="2"/>
       <c r="C124" s="2"/>
       <c r="D124" s="2"/>
       <c r="E124" s="5" t="s">
@@ -11172,10 +11173,10 @@
       </c>
     </row>
     <row r="125" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A125" s="13" t="s">
+      <c r="A125" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B125" s="13" t="s">
+      <c r="B125" s="2" t="s">
         <v>152</v>
       </c>
       <c r="C125" s="2" t="s">
@@ -11213,11 +11214,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="126" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A126" s="13" t="s">
+    <row r="126" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A126" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B126" s="13"/>
+      <c r="B126" s="2"/>
       <c r="C126" s="2"/>
       <c r="D126" s="2"/>
       <c r="E126" s="3" t="s">
@@ -11251,11 +11252,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="127" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A127" s="13" t="s">
+    <row r="127" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A127" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B127" s="13" t="s">
+      <c r="B127" s="2" t="s">
         <v>165</v>
       </c>
       <c r="C127" s="2" t="s">
@@ -11296,10 +11297,10 @@
       </c>
     </row>
     <row r="128" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A128" s="13" t="s">
+      <c r="A128" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B128" s="13" t="s">
+      <c r="B128" s="2" t="s">
         <v>151</v>
       </c>
       <c r="C128" s="2" t="s">
@@ -11339,11 +11340,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="129" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A129" s="13" t="s">
+    <row r="129" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A129" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B129" s="13"/>
+      <c r="B129" s="2"/>
       <c r="C129" s="2"/>
       <c r="D129" s="2"/>
       <c r="E129" s="3" t="s">
@@ -11377,11 +11378,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="130" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A130" s="13" t="s">
+    <row r="130" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A130" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B130" s="13" t="s">
+      <c r="B130" s="2" t="s">
         <v>232</v>
       </c>
       <c r="C130" s="2" t="s">
@@ -11422,10 +11423,10 @@
       </c>
     </row>
     <row r="131" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A131" s="13" t="s">
+      <c r="A131" s="2" t="s">
         <v>1716</v>
       </c>
-      <c r="B131" s="13" t="s">
+      <c r="B131" s="2" t="s">
         <v>278</v>
       </c>
       <c r="C131" s="12"/>
@@ -11460,10 +11461,10 @@
       <c r="P131" s="2"/>
     </row>
     <row r="132" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A132" s="13" t="s">
+      <c r="A132" s="2" t="s">
         <v>1717</v>
       </c>
-      <c r="B132" s="13" t="s">
+      <c r="B132" s="2" t="s">
         <v>279</v>
       </c>
       <c r="C132" s="12"/>
@@ -11498,10 +11499,10 @@
       <c r="P132" s="2"/>
     </row>
     <row r="133" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A133" s="13" t="s">
+      <c r="A133" s="2" t="s">
         <v>1718</v>
       </c>
-      <c r="B133" s="13" t="s">
+      <c r="B133" s="2" t="s">
         <v>280</v>
       </c>
       <c r="C133" s="12"/>
@@ -11536,10 +11537,10 @@
       <c r="P133" s="2"/>
     </row>
     <row r="134" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A134" s="13" t="s">
+      <c r="A134" s="2" t="s">
         <v>1719</v>
       </c>
-      <c r="B134" s="13" t="s">
+      <c r="B134" s="2" t="s">
         <v>281</v>
       </c>
       <c r="C134" s="12"/>
@@ -11574,10 +11575,10 @@
       <c r="P134" s="2"/>
     </row>
     <row r="135" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A135" s="13" t="s">
+      <c r="A135" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="B135" s="13" t="s">
+      <c r="B135" s="2" t="s">
         <v>273</v>
       </c>
       <c r="C135" s="2" t="s">
@@ -11618,10 +11619,10 @@
       </c>
     </row>
     <row r="136" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A136" s="13" t="s">
+      <c r="A136" s="2" t="s">
         <v>1650</v>
       </c>
-      <c r="B136" s="13" t="s">
+      <c r="B136" s="2" t="s">
         <v>270</v>
       </c>
       <c r="C136" s="12" t="s">
@@ -11660,10 +11661,10 @@
       <c r="P136" s="2"/>
     </row>
     <row r="137" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A137" s="13" t="s">
+      <c r="A137" s="2" t="s">
         <v>1651</v>
       </c>
-      <c r="B137" s="13" t="s">
+      <c r="B137" s="2" t="s">
         <v>271</v>
       </c>
       <c r="C137" s="12" t="s">
@@ -11700,10 +11701,10 @@
       <c r="P137" s="2"/>
     </row>
     <row r="138" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A138" s="13" t="s">
+      <c r="A138" s="2" t="s">
         <v>1652</v>
       </c>
-      <c r="B138" s="13" t="s">
+      <c r="B138" s="2" t="s">
         <v>272</v>
       </c>
       <c r="C138" s="12" t="s">
@@ -11739,11 +11740,11 @@
       <c r="O138" s="2"/>
       <c r="P138" s="2"/>
     </row>
-    <row r="139" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A139" s="13" t="s">
+    <row r="139" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A139" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="B139" s="13" t="s">
+      <c r="B139" s="2" t="s">
         <v>241</v>
       </c>
       <c r="C139" s="2" t="s">
@@ -11784,10 +11785,10 @@
       </c>
     </row>
     <row r="140" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A140" s="13" t="s">
+      <c r="A140" s="2" t="s">
         <v>1736</v>
       </c>
-      <c r="B140" s="13" t="s">
+      <c r="B140" s="2" t="s">
         <v>1737</v>
       </c>
       <c r="C140" s="12" t="s">
@@ -11824,10 +11825,10 @@
       <c r="P140" s="2"/>
     </row>
     <row r="141" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A141" s="13" t="s">
+      <c r="A141" s="2" t="s">
         <v>1734</v>
       </c>
-      <c r="B141" s="13" t="s">
+      <c r="B141" s="2" t="s">
         <v>1738</v>
       </c>
       <c r="C141" s="12" t="s">
@@ -11864,10 +11865,10 @@
       <c r="P141" s="2"/>
     </row>
     <row r="142" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A142" s="13" t="s">
+      <c r="A142" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B142" s="13" t="s">
+      <c r="B142" s="2" t="s">
         <v>290</v>
       </c>
       <c r="C142" s="2" t="s">
@@ -11908,10 +11909,10 @@
       </c>
     </row>
     <row r="143" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A143" s="13" t="s">
+      <c r="A143" s="2" t="s">
         <v>1711</v>
       </c>
-      <c r="B143" s="13" t="s">
+      <c r="B143" s="2" t="s">
         <v>344</v>
       </c>
       <c r="C143" s="2" t="s">
@@ -11937,10 +11938,10 @@
         <v>161</v>
       </c>
       <c r="K143" s="12"/>
-      <c r="L143" s="15" t="s">
+      <c r="L143" s="13" t="s">
         <v>1828</v>
       </c>
-      <c r="M143" s="15" t="s">
+      <c r="M143" s="13" t="s">
         <v>150</v>
       </c>
       <c r="N143" s="2"/>
@@ -11948,10 +11949,10 @@
       <c r="P143" s="2"/>
     </row>
     <row r="144" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A144" s="13" t="s">
+      <c r="A144" s="2" t="s">
         <v>1712</v>
       </c>
-      <c r="B144" s="13" t="s">
+      <c r="B144" s="2" t="s">
         <v>343</v>
       </c>
       <c r="C144" s="2" t="s">
@@ -11977,21 +11978,21 @@
         <v>161</v>
       </c>
       <c r="K144" s="12"/>
-      <c r="L144" s="15" t="s">
+      <c r="L144" s="13" t="s">
         <v>1827</v>
       </c>
-      <c r="M144" s="15" t="s">
+      <c r="M144" s="13" t="s">
         <v>150</v>
       </c>
       <c r="N144" s="2"/>
       <c r="O144" s="2"/>
       <c r="P144" s="2"/>
     </row>
-    <row r="145" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A145" s="13" t="s">
+    <row r="145" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A145" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B145" s="13" t="s">
+      <c r="B145" s="2" t="s">
         <v>154</v>
       </c>
       <c r="C145" s="2" t="s">
@@ -12029,11 +12030,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="146" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A146" s="13" t="s">
+    <row r="146" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A146" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B146" s="13" t="s">
+      <c r="B146" s="2" t="s">
         <v>155</v>
       </c>
       <c r="C146" s="2" t="s">
@@ -12071,11 +12072,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="147" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A147" s="13" t="s">
+    <row r="147" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A147" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B147" s="13" t="s">
+      <c r="B147" s="2" t="s">
         <v>237</v>
       </c>
       <c r="C147" s="2" t="s">
@@ -12114,10 +12115,10 @@
       </c>
     </row>
     <row r="148" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A148" s="13" t="s">
+      <c r="A148" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B148" s="13" t="s">
+      <c r="B148" s="2" t="s">
         <v>1837</v>
       </c>
       <c r="C148" s="2" t="s">
@@ -12158,29 +12159,29 @@
       </c>
     </row>
     <row r="149" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A149" s="15" t="s">
+      <c r="A149" s="13" t="s">
         <v>1834</v>
       </c>
-      <c r="B149" s="15" t="s">
+      <c r="B149" s="13" t="s">
         <v>1838</v>
       </c>
-      <c r="C149" s="15" t="s">
+      <c r="C149" s="13" t="s">
         <v>1638</v>
       </c>
-      <c r="D149" s="15"/>
-      <c r="E149" s="15"/>
-      <c r="F149" s="15"/>
-      <c r="G149" s="15"/>
-      <c r="H149" s="15"/>
-      <c r="I149" s="15"/>
+      <c r="D149" s="13"/>
+      <c r="E149" s="13"/>
+      <c r="F149" s="13"/>
+      <c r="G149" s="13"/>
+      <c r="H149" s="13"/>
+      <c r="I149" s="13"/>
       <c r="J149" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="K149" s="15"/>
-      <c r="L149" s="15" t="s">
+      <c r="K149" s="13"/>
+      <c r="L149" s="13" t="s">
         <v>1757</v>
       </c>
-      <c r="M149" s="15" t="s">
+      <c r="M149" s="13" t="s">
         <v>150</v>
       </c>
       <c r="N149" s="2"/>
@@ -12188,10 +12189,10 @@
       <c r="P149" s="5"/>
     </row>
     <row r="150" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A150" s="13" t="s">
+      <c r="A150" s="2" t="s">
         <v>1709</v>
       </c>
-      <c r="B150" s="13" t="s">
+      <c r="B150" s="2" t="s">
         <v>341</v>
       </c>
       <c r="C150" s="2" t="s">
@@ -12217,10 +12218,10 @@
         <v>161</v>
       </c>
       <c r="K150" s="12"/>
-      <c r="L150" s="15" t="s">
+      <c r="L150" s="13" t="s">
         <v>1832</v>
       </c>
-      <c r="M150" s="15" t="s">
+      <c r="M150" s="13" t="s">
         <v>150</v>
       </c>
       <c r="N150" s="2"/>
@@ -12228,10 +12229,10 @@
       <c r="P150" s="2"/>
     </row>
     <row r="151" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A151" s="13" t="s">
+      <c r="A151" s="2" t="s">
         <v>1653</v>
       </c>
-      <c r="B151" s="13" t="s">
+      <c r="B151" s="2" t="s">
         <v>274</v>
       </c>
       <c r="C151" s="12"/>
@@ -12265,11 +12266,11 @@
       <c r="O151" s="2"/>
       <c r="P151" s="2"/>
     </row>
-    <row r="152" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A152" s="13" t="s">
+    <row r="152" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A152" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B152" s="13" t="s">
+      <c r="B152" s="2" t="s">
         <v>1724</v>
       </c>
       <c r="C152" s="2" t="s">
@@ -12310,10 +12311,10 @@
       </c>
     </row>
     <row r="153" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A153" s="13" t="s">
+      <c r="A153" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="B153" s="13" t="s">
+      <c r="B153" s="2" t="s">
         <v>287</v>
       </c>
       <c r="C153" s="2" t="s">
@@ -12351,11 +12352,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="154" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A154" s="13" t="s">
+    <row r="154" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A154" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B154" s="13"/>
+      <c r="B154" s="2"/>
       <c r="C154" s="2"/>
       <c r="D154" s="2"/>
       <c r="E154" s="2"/>
@@ -12379,11 +12380,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="155" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A155" s="13" t="s">
+    <row r="155" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A155" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B155" s="13"/>
+      <c r="B155" s="2"/>
       <c r="C155" s="2"/>
       <c r="D155" s="2"/>
       <c r="E155" s="2"/>
@@ -12408,10 +12409,10 @@
       </c>
     </row>
     <row r="156" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A156" s="13" t="s">
+      <c r="A156" s="2" t="s">
         <v>1695</v>
       </c>
-      <c r="B156" s="13" t="s">
+      <c r="B156" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C156" s="2" t="s">
@@ -12437,10 +12438,10 @@
         <v>161</v>
       </c>
       <c r="K156" s="12"/>
-      <c r="L156" s="15" t="s">
+      <c r="L156" s="13" t="s">
         <v>1814</v>
       </c>
-      <c r="M156" s="15" t="s">
+      <c r="M156" s="13" t="s">
         <v>150</v>
       </c>
       <c r="N156" s="2"/>
@@ -12448,10 +12449,10 @@
       <c r="P156" s="2"/>
     </row>
     <row r="157" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A157" s="13" t="s">
+      <c r="A157" s="2" t="s">
         <v>1658</v>
       </c>
-      <c r="B157" s="13" t="s">
+      <c r="B157" s="2" t="s">
         <v>283</v>
       </c>
       <c r="C157" s="2" t="s">
@@ -12488,10 +12489,10 @@
       <c r="P157" s="2"/>
     </row>
     <row r="158" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A158" s="13" t="s">
+      <c r="A158" s="2" t="s">
         <v>1660</v>
       </c>
-      <c r="B158" s="13" t="s">
+      <c r="B158" s="2" t="s">
         <v>326</v>
       </c>
       <c r="C158" s="2" t="s">
@@ -12517,21 +12518,21 @@
         <v>161</v>
       </c>
       <c r="K158" s="12"/>
-      <c r="L158" s="15" t="s">
+      <c r="L158" s="13" t="s">
         <v>1813</v>
       </c>
-      <c r="M158" s="15" t="s">
+      <c r="M158" s="13" t="s">
         <v>150</v>
       </c>
       <c r="N158" s="2"/>
       <c r="O158" s="2"/>
       <c r="P158" s="2"/>
     </row>
-    <row r="159" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A159" s="13" t="s">
+    <row r="159" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A159" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B159" s="13" t="s">
+      <c r="B159" s="2" t="s">
         <v>156</v>
       </c>
       <c r="C159" s="2" t="s">
@@ -12571,11 +12572,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="160" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A160" s="13" t="s">
+    <row r="160" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A160" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B160" s="13" t="s">
+      <c r="B160" s="2" t="s">
         <v>157</v>
       </c>
       <c r="C160" s="2" t="s">
@@ -12615,11 +12616,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="161" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A161" s="13" t="s">
+    <row r="161" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A161" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B161" s="13" t="s">
+      <c r="B161" s="2" t="s">
         <v>229</v>
       </c>
       <c r="C161" s="2" t="s">
@@ -12658,10 +12659,10 @@
       </c>
     </row>
     <row r="162" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A162" s="13" t="s">
+      <c r="A162" s="2" t="s">
         <v>1644</v>
       </c>
-      <c r="B162" s="13" t="s">
+      <c r="B162" s="2" t="s">
         <v>266</v>
       </c>
       <c r="C162" s="12" t="s">
@@ -12700,10 +12701,10 @@
       <c r="P162" s="2"/>
     </row>
     <row r="163" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A163" s="13" t="s">
+      <c r="A163" s="2" t="s">
         <v>1685</v>
       </c>
-      <c r="B163" s="13" t="s">
+      <c r="B163" s="2" t="s">
         <v>314</v>
       </c>
       <c r="C163" s="12" t="s">
@@ -12741,11 +12742,11 @@
       <c r="O163" s="2"/>
       <c r="P163" s="2"/>
     </row>
-    <row r="164" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A164" s="13" t="s">
+    <row r="164" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A164" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B164" s="13"/>
+      <c r="B164" s="2"/>
       <c r="C164" s="2" t="s">
         <v>1641</v>
       </c>
@@ -12781,11 +12782,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="165" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A165" s="13" t="s">
+    <row r="165" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A165" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B165" s="13"/>
+      <c r="B165" s="2"/>
       <c r="C165" s="2" t="s">
         <v>1720</v>
       </c>
@@ -12821,11 +12822,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="166" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A166" s="13" t="s">
+    <row r="166" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A166" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="B166" s="13" t="s">
+      <c r="B166" s="2" t="s">
         <v>159</v>
       </c>
       <c r="C166" s="2" t="s">
@@ -12863,11 +12864,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="167" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A167" s="13" t="s">
+    <row r="167" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A167" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B167" s="13" t="s">
+      <c r="B167" s="2" t="s">
         <v>142</v>
       </c>
       <c r="C167" s="2" t="s">
@@ -12905,11 +12906,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="168" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A168" s="13" t="s">
+    <row r="168" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A168" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B168" s="13" t="s">
+      <c r="B168" s="2" t="s">
         <v>144</v>
       </c>
       <c r="C168" s="2" t="s">
@@ -12948,10 +12949,10 @@
       </c>
     </row>
     <row r="169" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A169" s="13" t="s">
+      <c r="A169" s="2" t="s">
         <v>1704</v>
       </c>
-      <c r="B169" s="13" t="s">
+      <c r="B169" s="2" t="s">
         <v>336</v>
       </c>
       <c r="C169" s="2" t="s">
@@ -12977,21 +12978,21 @@
         <v>161</v>
       </c>
       <c r="K169" s="12"/>
-      <c r="L169" s="15" t="s">
+      <c r="L169" s="13" t="s">
         <v>1821</v>
       </c>
-      <c r="M169" s="15" t="s">
+      <c r="M169" s="13" t="s">
         <v>150</v>
       </c>
       <c r="N169" s="2"/>
       <c r="O169" s="2"/>
       <c r="P169" s="2"/>
     </row>
-    <row r="170" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A170" s="13" t="s">
+    <row r="170" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A170" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B170" s="13"/>
+      <c r="B170" s="2"/>
       <c r="C170" s="2"/>
       <c r="D170" s="2"/>
       <c r="E170" s="2"/>
@@ -13016,10 +13017,10 @@
       </c>
     </row>
     <row r="171" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A171" s="13" t="s">
+      <c r="A171" s="2" t="s">
         <v>1713</v>
       </c>
-      <c r="B171" s="13" t="s">
+      <c r="B171" s="2" t="s">
         <v>345</v>
       </c>
       <c r="C171" s="2" t="s">
@@ -13045,10 +13046,10 @@
         <v>161</v>
       </c>
       <c r="K171" s="12"/>
-      <c r="L171" s="15" t="s">
+      <c r="L171" s="13" t="s">
         <v>1829</v>
       </c>
-      <c r="M171" s="15" t="s">
+      <c r="M171" s="13" t="s">
         <v>150</v>
       </c>
       <c r="N171" s="2"/>
@@ -13056,10 +13057,10 @@
       <c r="P171" s="2"/>
     </row>
     <row r="172" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A172" s="13" t="s">
+      <c r="A172" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B172" s="13" t="s">
+      <c r="B172" s="2" t="s">
         <v>231</v>
       </c>
       <c r="C172" s="2" t="s">
@@ -13103,11 +13104,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="173" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A173" s="13" t="s">
+    <row r="173" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A173" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B173" s="13"/>
+      <c r="B173" s="2"/>
       <c r="C173" s="2"/>
       <c r="D173" s="2"/>
       <c r="E173" s="2"/>
@@ -13131,11 +13132,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="174" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A174" s="13" t="s">
+    <row r="174" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A174" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B174" s="13"/>
+      <c r="B174" s="2"/>
       <c r="C174" s="2"/>
       <c r="D174" s="2"/>
       <c r="E174" s="3" t="s">
@@ -13169,11 +13170,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="175" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A175" s="13" t="s">
+    <row r="175" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A175" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B175" s="13" t="s">
+      <c r="B175" s="2" t="s">
         <v>202</v>
       </c>
       <c r="C175" s="2" t="s">
@@ -13213,11 +13214,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="176" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A176" s="13" t="s">
+    <row r="176" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A176" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B176" s="13" t="s">
+      <c r="B176" s="2" t="s">
         <v>203</v>
       </c>
       <c r="C176" s="2" t="s">
@@ -13257,11 +13258,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="177" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A177" s="13" t="s">
+    <row r="177" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A177" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B177" s="13" t="s">
+      <c r="B177" s="2" t="s">
         <v>204</v>
       </c>
       <c r="C177" s="2" t="s">
@@ -13301,11 +13302,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="178" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A178" s="13" t="s">
+    <row r="178" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A178" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B178" s="13" t="s">
+      <c r="B178" s="2" t="s">
         <v>205</v>
       </c>
       <c r="C178" s="2" t="s">
@@ -13345,11 +13346,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="179" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A179" s="13" t="s">
+    <row r="179" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A179" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B179" s="13" t="s">
+      <c r="B179" s="2" t="s">
         <v>206</v>
       </c>
       <c r="C179" s="2" t="s">
@@ -13389,11 +13390,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="180" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A180" s="13" t="s">
+    <row r="180" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A180" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B180" s="13" t="s">
+      <c r="B180" s="2" t="s">
         <v>207</v>
       </c>
       <c r="C180" s="2" t="s">
@@ -13433,11 +13434,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="181" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A181" s="13" t="s">
+    <row r="181" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A181" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B181" s="13" t="s">
+      <c r="B181" s="2" t="s">
         <v>208</v>
       </c>
       <c r="C181" s="2" t="s">
@@ -13477,11 +13478,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="182" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A182" s="13" t="s">
+    <row r="182" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A182" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B182" s="13" t="s">
+      <c r="B182" s="2" t="s">
         <v>209</v>
       </c>
       <c r="C182" s="2" t="s">
@@ -13521,11 +13522,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="183" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A183" s="13" t="s">
+    <row r="183" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A183" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B183" s="13" t="s">
+      <c r="B183" s="2" t="s">
         <v>210</v>
       </c>
       <c r="C183" s="2" t="s">
@@ -13565,11 +13566,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="184" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A184" s="13" t="s">
+    <row r="184" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A184" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B184" s="13" t="s">
+      <c r="B184" s="2" t="s">
         <v>211</v>
       </c>
       <c r="C184" s="2" t="s">
@@ -13609,11 +13610,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="185" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A185" s="13" t="s">
+    <row r="185" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A185" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B185" s="13" t="s">
+      <c r="B185" s="2" t="s">
         <v>212</v>
       </c>
       <c r="C185" s="2" t="s">
@@ -13653,11 +13654,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="186" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A186" s="13" t="s">
+    <row r="186" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A186" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B186" s="13" t="s">
+      <c r="B186" s="2" t="s">
         <v>213</v>
       </c>
       <c r="C186" s="2" t="s">
@@ -13697,11 +13698,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="187" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A187" s="13" t="s">
+    <row r="187" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A187" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B187" s="13" t="s">
+      <c r="B187" s="2" t="s">
         <v>214</v>
       </c>
       <c r="C187" s="2" t="s">
@@ -13741,11 +13742,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="188" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A188" s="13" t="s">
+    <row r="188" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A188" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B188" s="13" t="s">
+      <c r="B188" s="2" t="s">
         <v>215</v>
       </c>
       <c r="C188" s="2" t="s">
@@ -13785,11 +13786,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="189" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A189" s="13" t="s">
+    <row r="189" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A189" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B189" s="13" t="s">
+      <c r="B189" s="2" t="s">
         <v>216</v>
       </c>
       <c r="C189" s="2" t="s">
@@ -13829,11 +13830,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="190" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A190" s="13" t="s">
+    <row r="190" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A190" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B190" s="13" t="s">
+      <c r="B190" s="2" t="s">
         <v>217</v>
       </c>
       <c r="C190" s="2" t="s">
@@ -13873,11 +13874,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="191" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A191" s="13" t="s">
+    <row r="191" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A191" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B191" s="13"/>
+      <c r="B191" s="2"/>
       <c r="C191" s="2"/>
       <c r="D191" s="2"/>
       <c r="E191" s="2"/>
@@ -13902,10 +13903,10 @@
       </c>
     </row>
     <row r="192" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A192" s="13" t="s">
+      <c r="A192" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B192" s="13" t="s">
+      <c r="B192" s="2" t="s">
         <v>167</v>
       </c>
       <c r="C192" s="2" t="s">
@@ -13950,10 +13951,10 @@
       </c>
     </row>
     <row r="193" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A193" s="13" t="s">
+      <c r="A193" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B193" s="13" t="s">
+      <c r="B193" s="2" t="s">
         <v>288</v>
       </c>
       <c r="C193" s="2" t="s">
@@ -13992,10 +13993,10 @@
       </c>
     </row>
     <row r="194" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A194" s="13" t="s">
+      <c r="A194" s="2" t="s">
         <v>1784</v>
       </c>
-      <c r="B194" s="13" t="s">
+      <c r="B194" s="2" t="s">
         <v>300</v>
       </c>
       <c r="C194" s="12" t="s">
@@ -14031,11 +14032,11 @@
       <c r="O194" s="2"/>
       <c r="P194" s="2"/>
     </row>
-    <row r="195" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A195" s="13" t="s">
+    <row r="195" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A195" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B195" s="13" t="s">
+      <c r="B195" s="2" t="s">
         <v>143</v>
       </c>
       <c r="C195" s="2" t="s">
@@ -14074,10 +14075,10 @@
       </c>
     </row>
     <row r="196" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A196" s="13" t="s">
+      <c r="A196" s="2" t="s">
         <v>1680</v>
       </c>
-      <c r="B196" s="13" t="s">
+      <c r="B196" s="2" t="s">
         <v>295</v>
       </c>
       <c r="C196" s="12" t="s">
@@ -14114,10 +14115,10 @@
       <c r="P196" s="2"/>
     </row>
     <row r="197" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A197" s="13" t="s">
+      <c r="A197" s="2" t="s">
         <v>1681</v>
       </c>
-      <c r="B197" s="13" t="s">
+      <c r="B197" s="2" t="s">
         <v>296</v>
       </c>
       <c r="C197" s="12" t="s">
@@ -14154,10 +14155,10 @@
       <c r="P197" s="2"/>
     </row>
     <row r="198" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A198" s="13" t="s">
+      <c r="A198" s="2" t="s">
         <v>1706</v>
       </c>
-      <c r="B198" s="13" t="s">
+      <c r="B198" s="2" t="s">
         <v>338</v>
       </c>
       <c r="C198" s="2" t="s">
@@ -14183,21 +14184,21 @@
         <v>161</v>
       </c>
       <c r="K198" s="12"/>
-      <c r="L198" s="15" t="s">
+      <c r="L198" s="13" t="s">
         <v>1823</v>
       </c>
-      <c r="M198" s="15" t="s">
+      <c r="M198" s="13" t="s">
         <v>150</v>
       </c>
       <c r="N198" s="2"/>
       <c r="O198" s="2"/>
       <c r="P198" s="2"/>
     </row>
-    <row r="199" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A199" s="13" t="s">
+    <row r="199" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A199" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B199" s="13"/>
+      <c r="B199" s="2"/>
       <c r="C199" s="2"/>
       <c r="D199" s="2"/>
       <c r="E199" s="2"/>
@@ -14221,11 +14222,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="200" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A200" s="13" t="s">
+    <row r="200" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A200" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B200" s="13" t="s">
+      <c r="B200" s="2" t="s">
         <v>160</v>
       </c>
       <c r="C200" s="2" t="s">
@@ -14264,10 +14265,10 @@
       </c>
     </row>
     <row r="201" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A201" s="13" t="s">
+      <c r="A201" s="2" t="s">
         <v>1707</v>
       </c>
-      <c r="B201" s="13" t="s">
+      <c r="B201" s="2" t="s">
         <v>340</v>
       </c>
       <c r="C201" s="2" t="s">
@@ -14293,10 +14294,10 @@
         <v>161</v>
       </c>
       <c r="K201" s="12"/>
-      <c r="L201" s="15" t="s">
+      <c r="L201" s="13" t="s">
         <v>1825</v>
       </c>
-      <c r="M201" s="15" t="s">
+      <c r="M201" s="13" t="s">
         <v>150</v>
       </c>
       <c r="N201" s="2"/>
@@ -14304,10 +14305,10 @@
       <c r="P201" s="2"/>
     </row>
     <row r="202" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A202" s="13" t="s">
+      <c r="A202" s="2" t="s">
         <v>1708</v>
       </c>
-      <c r="B202" s="13" t="s">
+      <c r="B202" s="2" t="s">
         <v>339</v>
       </c>
       <c r="C202" s="2" t="s">
@@ -14333,10 +14334,10 @@
         <v>161</v>
       </c>
       <c r="K202" s="12"/>
-      <c r="L202" s="15" t="s">
+      <c r="L202" s="13" t="s">
         <v>1824</v>
       </c>
-      <c r="M202" s="15" t="s">
+      <c r="M202" s="13" t="s">
         <v>150</v>
       </c>
       <c r="N202" s="2"/>
@@ -14344,10 +14345,10 @@
       <c r="P202" s="2"/>
     </row>
     <row r="203" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A203" s="13" t="s">
+      <c r="A203" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B203" s="13" t="s">
+      <c r="B203" s="2" t="s">
         <v>168</v>
       </c>
       <c r="C203" s="2" t="s">
@@ -14388,10 +14389,10 @@
       </c>
     </row>
     <row r="204" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A204" s="13" t="s">
+      <c r="A204" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B204" s="13" t="s">
+      <c r="B204" s="2" t="s">
         <v>291</v>
       </c>
       <c r="C204" s="2" t="s">
@@ -14432,10 +14433,10 @@
       </c>
     </row>
     <row r="205" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A205" s="13" t="s">
+      <c r="A205" s="2" t="s">
         <v>1698</v>
       </c>
-      <c r="B205" s="13" t="s">
+      <c r="B205" s="2" t="s">
         <v>330</v>
       </c>
       <c r="C205" s="2" t="s">
@@ -14461,10 +14462,10 @@
         <v>161</v>
       </c>
       <c r="K205" s="12"/>
-      <c r="L205" s="15" t="s">
+      <c r="L205" s="13" t="s">
         <v>1817</v>
       </c>
-      <c r="M205" s="15" t="s">
+      <c r="M205" s="13" t="s">
         <v>150</v>
       </c>
       <c r="N205" s="2"/>
@@ -14472,10 +14473,10 @@
       <c r="P205" s="2"/>
     </row>
     <row r="206" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A206" s="13" t="s">
+      <c r="A206" s="2" t="s">
         <v>1802</v>
       </c>
-      <c r="B206" s="13" t="s">
+      <c r="B206" s="2" t="s">
         <v>315</v>
       </c>
       <c r="C206" s="12" t="s">
@@ -14512,10 +14513,10 @@
       <c r="P206" s="2"/>
     </row>
     <row r="207" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A207" s="13" t="s">
+      <c r="A207" s="2" t="s">
         <v>1654</v>
       </c>
-      <c r="B207" s="13" t="s">
+      <c r="B207" s="2" t="s">
         <v>275</v>
       </c>
       <c r="C207" s="12"/>
@@ -14550,10 +14551,10 @@
       <c r="P207" s="2"/>
     </row>
     <row r="208" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A208" s="13" t="s">
+      <c r="A208" s="2" t="s">
         <v>1664</v>
       </c>
-      <c r="B208" s="13" t="s">
+      <c r="B208" s="2" t="s">
         <v>277</v>
       </c>
       <c r="C208" s="12"/>
@@ -14587,11 +14588,11 @@
       <c r="O208" s="2"/>
       <c r="P208" s="2"/>
     </row>
-    <row r="209" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A209" s="13" t="s">
+    <row r="209" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A209" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="B209" s="13"/>
+      <c r="B209" s="2"/>
       <c r="C209" s="2"/>
       <c r="D209" s="2"/>
       <c r="E209" s="5" t="s">
@@ -14625,11 +14626,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="210" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A210" s="13" t="s">
+    <row r="210" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A210" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B210" s="13" t="s">
+      <c r="B210" s="2" t="s">
         <v>230</v>
       </c>
       <c r="C210" s="2" t="s">
@@ -14668,10 +14669,10 @@
       </c>
     </row>
     <row r="211" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A211" s="13" t="s">
+      <c r="A211" s="2" t="s">
         <v>1661</v>
       </c>
-      <c r="B211" s="13" t="s">
+      <c r="B211" s="2" t="s">
         <v>284</v>
       </c>
       <c r="C211" s="12" t="s">
@@ -14707,11 +14708,11 @@
       <c r="O211" s="2"/>
       <c r="P211" s="2"/>
     </row>
-    <row r="212" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A212" s="13" t="s">
+    <row r="212" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A212" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B212" s="13"/>
+      <c r="B212" s="2"/>
       <c r="C212" s="2"/>
       <c r="D212" s="2"/>
       <c r="E212" s="5" t="s">
@@ -14752,10 +14753,10 @@
       </c>
     </row>
     <row r="213" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A213" s="13" t="s">
+      <c r="A213" s="2" t="s">
         <v>1647</v>
       </c>
-      <c r="B213" s="13" t="s">
+      <c r="B213" s="2" t="s">
         <v>264</v>
       </c>
       <c r="C213" s="12" t="s">
@@ -14792,10 +14793,10 @@
       <c r="P213" s="2"/>
     </row>
     <row r="214" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A214" s="13" t="s">
+      <c r="A214" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B214" s="13" t="s">
+      <c r="B214" s="2" t="s">
         <v>169</v>
       </c>
       <c r="C214" s="2" t="s">
@@ -14836,10 +14837,10 @@
       </c>
     </row>
     <row r="215" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A215" s="13" t="s">
+      <c r="A215" s="2" t="s">
         <v>1649</v>
       </c>
-      <c r="B215" s="13" t="s">
+      <c r="B215" s="2" t="s">
         <v>269</v>
       </c>
       <c r="C215" s="12" t="s">
@@ -14876,10 +14877,10 @@
       <c r="P215" s="2"/>
     </row>
     <row r="216" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A216" s="13" t="s">
+      <c r="A216" s="2" t="s">
         <v>1648</v>
       </c>
-      <c r="B216" s="13" t="s">
+      <c r="B216" s="2" t="s">
         <v>268</v>
       </c>
       <c r="C216" s="12" t="s">
@@ -14916,10 +14917,10 @@
       <c r="P216" s="2"/>
     </row>
     <row r="217" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A217" s="13" t="s">
+      <c r="A217" s="2" t="s">
         <v>1662</v>
       </c>
-      <c r="B217" s="13" t="s">
+      <c r="B217" s="2" t="s">
         <v>285</v>
       </c>
       <c r="C217" s="12" t="s">
@@ -14956,10 +14957,10 @@
       <c r="P217" s="2"/>
     </row>
     <row r="218" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A218" s="13" t="s">
+      <c r="A218" s="2" t="s">
         <v>1663</v>
       </c>
-      <c r="B218" s="13" t="s">
+      <c r="B218" s="2" t="s">
         <v>286</v>
       </c>
       <c r="C218" s="12" t="s">
@@ -14996,14 +14997,14 @@
       <c r="P218" s="2"/>
     </row>
     <row r="219" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A219" s="15" t="s">
+      <c r="A219" s="13" t="s">
         <v>1835</v>
       </c>
-      <c r="B219" s="18" t="s">
+      <c r="B219" s="16" t="s">
         <v>1767</v>
       </c>
-      <c r="C219" s="15"/>
-      <c r="D219" s="15"/>
+      <c r="C219" s="13"/>
+      <c r="D219" s="13"/>
       <c r="E219" s="5" t="s">
         <v>161</v>
       </c>
@@ -15019,12 +15020,12 @@
       <c r="I219" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="J219" s="15"/>
-      <c r="K219" s="15"/>
-      <c r="L219" s="18" t="s">
+      <c r="J219" s="13"/>
+      <c r="K219" s="13"/>
+      <c r="L219" s="16" t="s">
         <v>1767</v>
       </c>
-      <c r="M219" s="15" t="s">
+      <c r="M219" s="13" t="s">
         <v>150</v>
       </c>
       <c r="N219" s="2"/>
@@ -15032,14 +15033,14 @@
       <c r="P219" s="2"/>
     </row>
     <row r="220" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A220" s="18" t="s">
+      <c r="A220" s="16" t="s">
         <v>1836</v>
       </c>
-      <c r="B220" s="18" t="s">
+      <c r="B220" s="16" t="s">
         <v>1768</v>
       </c>
-      <c r="C220" s="18"/>
-      <c r="D220" s="18"/>
+      <c r="C220" s="16"/>
+      <c r="D220" s="16"/>
       <c r="E220" s="5" t="s">
         <v>161</v>
       </c>
@@ -15055,688 +15056,143 @@
       <c r="I220" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="J220" s="18"/>
-      <c r="K220" s="18"/>
-      <c r="L220" s="18" t="s">
+      <c r="J220" s="16"/>
+      <c r="K220" s="16"/>
+      <c r="L220" s="16" t="s">
         <v>1768</v>
       </c>
-      <c r="M220" s="19" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="221" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A221" s="14"/>
-      <c r="B221" s="14"/>
-    </row>
-    <row r="222" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A222" s="14"/>
-      <c r="B222" s="14"/>
-    </row>
+      <c r="M220" s="17" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="221" spans="1:16" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="223" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A223" s="20" t="s">
+      <c r="A223" s="16" t="s">
         <v>1839</v>
       </c>
     </row>
     <row r="224" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A224" s="21" t="s">
+      <c r="A224" s="18" t="s">
         <v>1840</v>
       </c>
     </row>
-    <row r="225" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A225" s="17" t="s">
+    <row r="225" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A225" s="15" t="s">
         <v>1841</v>
       </c>
-      <c r="B225" s="14"/>
-    </row>
-    <row r="226" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A226" s="14"/>
-      <c r="B226" s="14"/>
-    </row>
-    <row r="227" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A227" s="14"/>
-      <c r="B227" s="14"/>
-    </row>
-    <row r="228" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A228" s="14"/>
-      <c r="B228" s="14"/>
-    </row>
-    <row r="229" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A229" s="14"/>
-      <c r="B229" s="14"/>
-    </row>
-    <row r="230" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A230" s="14"/>
-      <c r="B230" s="14"/>
-    </row>
-    <row r="231" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A231" s="14"/>
-      <c r="B231" s="14"/>
-    </row>
-    <row r="232" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A232" s="14"/>
-      <c r="B232" s="14"/>
-    </row>
-    <row r="233" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A233" s="14"/>
-      <c r="B233" s="14"/>
-    </row>
-    <row r="234" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A234" s="14"/>
-      <c r="B234" s="14"/>
-    </row>
-    <row r="235" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A235" s="14"/>
-      <c r="B235" s="14"/>
-    </row>
-    <row r="236" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A236" s="14"/>
-      <c r="B236" s="14"/>
-    </row>
-    <row r="237" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A237" s="14"/>
-      <c r="B237" s="14"/>
-    </row>
-    <row r="238" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A238" s="14"/>
-      <c r="B238" s="14"/>
-    </row>
-    <row r="239" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A239" s="14"/>
-      <c r="B239" s="14"/>
-    </row>
-    <row r="240" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A240" s="14"/>
-      <c r="B240" s="14"/>
-    </row>
-    <row r="241" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A241" s="14"/>
-      <c r="B241" s="14"/>
-    </row>
-    <row r="242" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A242" s="14"/>
-      <c r="B242" s="14"/>
-    </row>
-    <row r="243" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A243" s="14"/>
-      <c r="B243" s="14"/>
-    </row>
-    <row r="244" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A244" s="14"/>
-      <c r="B244" s="14"/>
-    </row>
-    <row r="245" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A245" s="14"/>
-      <c r="B245" s="14"/>
-    </row>
-    <row r="246" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A246" s="14"/>
-      <c r="B246" s="14"/>
-    </row>
-    <row r="247" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A247" s="14"/>
-      <c r="B247" s="14"/>
-    </row>
-    <row r="248" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A248" s="14"/>
-      <c r="B248" s="14"/>
-    </row>
-    <row r="249" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A249" s="14"/>
-      <c r="B249" s="14"/>
-    </row>
-    <row r="250" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A250" s="14"/>
-      <c r="B250" s="14"/>
-    </row>
-    <row r="251" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A251" s="14"/>
-      <c r="B251" s="14"/>
-    </row>
-    <row r="252" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A252" s="14"/>
-      <c r="B252" s="14"/>
-    </row>
-    <row r="253" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A253" s="14"/>
-      <c r="B253" s="14"/>
-    </row>
-    <row r="254" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A254" s="14"/>
-      <c r="B254" s="14"/>
-    </row>
-    <row r="255" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A255" s="14"/>
-      <c r="B255" s="14"/>
-    </row>
-    <row r="256" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A256" s="14"/>
-      <c r="B256" s="14"/>
-    </row>
-    <row r="257" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A257" s="14"/>
-      <c r="B257" s="14"/>
-    </row>
-    <row r="258" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A258" s="14"/>
-      <c r="B258" s="14"/>
-    </row>
-    <row r="259" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A259" s="14"/>
-      <c r="B259" s="14"/>
-    </row>
-    <row r="260" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A260" s="14"/>
-      <c r="B260" s="14"/>
-    </row>
-    <row r="261" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A261" s="14"/>
-      <c r="B261" s="14"/>
-    </row>
-    <row r="262" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A262" s="14"/>
-      <c r="B262" s="14"/>
-    </row>
-    <row r="263" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A263" s="14"/>
-      <c r="B263" s="14"/>
-    </row>
-    <row r="264" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A264" s="14"/>
-      <c r="B264" s="14"/>
-    </row>
-    <row r="265" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A265" s="14"/>
-      <c r="B265" s="14"/>
-    </row>
-    <row r="266" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A266" s="14"/>
-      <c r="B266" s="14"/>
-    </row>
-    <row r="267" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A267" s="14"/>
-      <c r="B267" s="14"/>
-    </row>
-    <row r="268" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A268" s="14"/>
-      <c r="B268" s="14"/>
-    </row>
-    <row r="269" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A269" s="14"/>
-      <c r="B269" s="14"/>
-    </row>
-    <row r="270" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A270" s="14"/>
-      <c r="B270" s="14"/>
-    </row>
-    <row r="271" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A271" s="14"/>
-      <c r="B271" s="14"/>
-    </row>
-    <row r="272" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A272" s="14"/>
-      <c r="B272" s="14"/>
-    </row>
-    <row r="273" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A273" s="14"/>
-      <c r="B273" s="14"/>
-    </row>
-    <row r="274" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A274" s="14"/>
-      <c r="B274" s="14"/>
-    </row>
-    <row r="275" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A275" s="14"/>
-      <c r="B275" s="14"/>
-    </row>
-    <row r="276" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A276" s="14"/>
-      <c r="B276" s="14"/>
-    </row>
-    <row r="277" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A277" s="14"/>
-      <c r="B277" s="14"/>
-    </row>
-    <row r="278" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A278" s="14"/>
-      <c r="B278" s="14"/>
-    </row>
-    <row r="279" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A279" s="14"/>
-      <c r="B279" s="14"/>
-    </row>
-    <row r="280" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A280" s="14"/>
-      <c r="B280" s="14"/>
-    </row>
-    <row r="281" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A281" s="14"/>
-      <c r="B281" s="14"/>
-    </row>
-    <row r="282" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A282" s="14"/>
-      <c r="B282" s="14"/>
-    </row>
-    <row r="283" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A283" s="14"/>
-      <c r="B283" s="14"/>
-    </row>
-    <row r="284" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A284" s="14"/>
-      <c r="B284" s="14"/>
-    </row>
-    <row r="285" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A285" s="14"/>
-      <c r="B285" s="14"/>
-    </row>
-    <row r="286" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A286" s="14"/>
-      <c r="B286" s="14"/>
-    </row>
-    <row r="287" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A287" s="14"/>
-      <c r="B287" s="14"/>
-    </row>
-    <row r="288" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A288" s="14"/>
-      <c r="B288" s="14"/>
-    </row>
-    <row r="289" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A289" s="14"/>
-      <c r="B289" s="14"/>
-    </row>
-    <row r="290" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A290" s="14"/>
-      <c r="B290" s="14"/>
-    </row>
-    <row r="291" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A291" s="14"/>
-      <c r="B291" s="14"/>
-    </row>
-    <row r="292" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A292" s="14"/>
-      <c r="B292" s="14"/>
-    </row>
-    <row r="293" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A293" s="14"/>
-      <c r="B293" s="14"/>
-    </row>
-    <row r="294" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A294" s="14"/>
-      <c r="B294" s="14"/>
-    </row>
-    <row r="295" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A295" s="14"/>
-      <c r="B295" s="14"/>
-    </row>
-    <row r="296" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A296" s="14"/>
-      <c r="B296" s="14"/>
-    </row>
-    <row r="297" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A297" s="14"/>
-      <c r="B297" s="14"/>
-    </row>
-    <row r="298" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A298" s="14"/>
-      <c r="B298" s="14"/>
-    </row>
-    <row r="299" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A299" s="14"/>
-      <c r="B299" s="14"/>
-    </row>
-    <row r="300" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A300" s="14"/>
-      <c r="B300" s="14"/>
-    </row>
-    <row r="301" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A301" s="14"/>
-      <c r="B301" s="14"/>
-    </row>
-    <row r="302" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A302" s="14"/>
-      <c r="B302" s="14"/>
-    </row>
-    <row r="303" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A303" s="14"/>
-      <c r="B303" s="14"/>
-    </row>
-    <row r="304" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A304" s="14"/>
-      <c r="B304" s="14"/>
-    </row>
-    <row r="305" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A305" s="14"/>
-      <c r="B305" s="14"/>
-    </row>
-    <row r="306" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A306" s="14"/>
-      <c r="B306" s="14"/>
-    </row>
-    <row r="307" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A307" s="14"/>
-      <c r="B307" s="14"/>
-    </row>
-    <row r="308" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A308" s="14"/>
-      <c r="B308" s="14"/>
-    </row>
-    <row r="309" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A309" s="14"/>
-      <c r="B309" s="14"/>
-    </row>
-    <row r="310" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A310" s="14"/>
-      <c r="B310" s="14"/>
-    </row>
-    <row r="311" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A311" s="14"/>
-      <c r="B311" s="14"/>
-    </row>
-    <row r="312" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A312" s="14"/>
-      <c r="B312" s="14"/>
-    </row>
-    <row r="313" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A313" s="14"/>
-      <c r="B313" s="14"/>
-    </row>
-    <row r="314" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A314" s="14"/>
-      <c r="B314" s="14"/>
-    </row>
-    <row r="315" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A315" s="14"/>
-      <c r="B315" s="14"/>
-    </row>
-    <row r="316" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A316" s="14"/>
-      <c r="B316" s="14"/>
-    </row>
-    <row r="317" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A317" s="14"/>
-      <c r="B317" s="14"/>
-    </row>
-    <row r="318" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A318" s="14"/>
-      <c r="B318" s="14"/>
-    </row>
-    <row r="319" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A319" s="14"/>
-      <c r="B319" s="14"/>
-    </row>
-    <row r="320" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A320" s="14"/>
-      <c r="B320" s="14"/>
-    </row>
-    <row r="321" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A321" s="14"/>
-      <c r="B321" s="14"/>
-    </row>
-    <row r="322" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A322" s="14"/>
-      <c r="B322" s="14"/>
-    </row>
-    <row r="323" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A323" s="14"/>
-      <c r="B323" s="14"/>
-    </row>
-    <row r="324" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A324" s="14"/>
-      <c r="B324" s="14"/>
-    </row>
-    <row r="325" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A325" s="14"/>
-      <c r="B325" s="14"/>
-    </row>
-    <row r="326" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A326" s="14"/>
-      <c r="B326" s="14"/>
-    </row>
-    <row r="327" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A327" s="14"/>
-      <c r="B327" s="14"/>
-    </row>
-    <row r="328" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A328" s="14"/>
-      <c r="B328" s="14"/>
-    </row>
-    <row r="329" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A329" s="14"/>
-      <c r="B329" s="14"/>
-    </row>
-    <row r="330" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A330" s="14"/>
-      <c r="B330" s="14"/>
-    </row>
-    <row r="331" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A331" s="14"/>
-      <c r="B331" s="14"/>
-    </row>
-    <row r="332" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A332" s="14"/>
-      <c r="B332" s="14"/>
-    </row>
-    <row r="333" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A333" s="14"/>
-      <c r="B333" s="14"/>
-    </row>
-    <row r="334" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A334" s="14"/>
-      <c r="B334" s="14"/>
-    </row>
-    <row r="335" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A335" s="14"/>
-      <c r="B335" s="14"/>
-    </row>
-    <row r="336" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A336" s="14"/>
-      <c r="B336" s="14"/>
-    </row>
-    <row r="337" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A337" s="14"/>
-      <c r="B337" s="14"/>
-    </row>
-    <row r="338" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A338" s="14"/>
-      <c r="B338" s="14"/>
-    </row>
-    <row r="339" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A339" s="14"/>
-      <c r="B339" s="14"/>
-    </row>
-    <row r="340" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A340" s="14"/>
-      <c r="B340" s="14"/>
-    </row>
-    <row r="341" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A341" s="14"/>
-      <c r="B341" s="14"/>
-    </row>
-    <row r="342" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A342" s="14"/>
-      <c r="B342" s="14"/>
-    </row>
-    <row r="343" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A343" s="14"/>
-      <c r="B343" s="14"/>
-    </row>
-    <row r="344" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A344" s="14"/>
-      <c r="B344" s="14"/>
-    </row>
-    <row r="345" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A345" s="14"/>
-      <c r="B345" s="14"/>
-    </row>
-    <row r="346" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A346" s="14"/>
-      <c r="B346" s="14"/>
-    </row>
-    <row r="347" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A347" s="14"/>
-      <c r="B347" s="14"/>
-    </row>
-    <row r="348" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A348" s="14"/>
-      <c r="B348" s="14"/>
-    </row>
-    <row r="349" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A349" s="14"/>
-      <c r="B349" s="14"/>
-    </row>
-    <row r="350" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A350" s="14"/>
-      <c r="B350" s="14"/>
-    </row>
-    <row r="351" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A351" s="14"/>
-      <c r="B351" s="14"/>
-    </row>
-    <row r="352" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A352" s="14"/>
-      <c r="B352" s="14"/>
-    </row>
-    <row r="353" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A353" s="14"/>
-      <c r="B353" s="14"/>
-    </row>
-    <row r="354" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A354" s="14"/>
-      <c r="B354" s="14"/>
-    </row>
-    <row r="355" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A355" s="14"/>
-      <c r="B355" s="14"/>
-    </row>
-    <row r="356" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A356" s="14"/>
-      <c r="B356" s="14"/>
-    </row>
-    <row r="357" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A357" s="14"/>
-      <c r="B357" s="14"/>
-    </row>
-    <row r="358" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A358" s="14"/>
-      <c r="B358" s="14"/>
-    </row>
-    <row r="359" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A359" s="14"/>
-      <c r="B359" s="14"/>
-    </row>
-    <row r="360" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A360" s="14"/>
-      <c r="B360" s="14"/>
-    </row>
-    <row r="361" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A361" s="14"/>
-      <c r="B361" s="14"/>
-    </row>
-    <row r="362" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A362" s="14"/>
-      <c r="B362" s="14"/>
-    </row>
-    <row r="363" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A363" s="14"/>
-      <c r="B363" s="14"/>
-    </row>
-    <row r="364" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A364" s="14"/>
-      <c r="B364" s="14"/>
-    </row>
-    <row r="365" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A365" s="14"/>
-      <c r="B365" s="14"/>
-    </row>
-    <row r="366" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A366" s="14"/>
-      <c r="B366" s="14"/>
-    </row>
-    <row r="367" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A367" s="14"/>
-      <c r="B367" s="14"/>
-    </row>
-    <row r="368" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A368" s="14"/>
-      <c r="B368" s="14"/>
-    </row>
-    <row r="369" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A369" s="14"/>
-      <c r="B369" s="14"/>
-    </row>
-    <row r="370" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A370" s="14"/>
-      <c r="B370" s="14"/>
-    </row>
-    <row r="371" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A371" s="14"/>
-      <c r="B371" s="14"/>
-    </row>
-    <row r="372" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A372" s="14"/>
-      <c r="B372" s="14"/>
-    </row>
-    <row r="373" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A373" s="14"/>
-      <c r="B373" s="14"/>
-    </row>
-    <row r="374" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A374" s="14"/>
-      <c r="B374" s="14"/>
-    </row>
-    <row r="375" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A375" s="14"/>
-      <c r="B375" s="14"/>
-    </row>
-    <row r="376" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A376" s="14"/>
-      <c r="B376" s="14"/>
-    </row>
-    <row r="377" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A377" s="14"/>
-      <c r="B377" s="14"/>
-    </row>
-    <row r="378" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A378" s="14"/>
-      <c r="B378" s="14"/>
-    </row>
-    <row r="379" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A379" s="14"/>
-      <c r="B379" s="14"/>
-    </row>
-    <row r="380" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A380" s="14"/>
-      <c r="B380" s="14"/>
-    </row>
-    <row r="381" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A381" s="14"/>
-      <c r="B381" s="14"/>
-    </row>
-    <row r="382" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A382" s="14"/>
-      <c r="B382" s="14"/>
-    </row>
-    <row r="383" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A383" s="14"/>
-      <c r="B383" s="14"/>
-    </row>
-    <row r="384" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A384" s="14"/>
-      <c r="B384" s="14"/>
-    </row>
-    <row r="385" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A385" s="14"/>
-      <c r="B385" s="14"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P221"/>
+  <autoFilter ref="A1:P221" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <filterColumn colId="11">
+      <filters>
+        <filter val="Accelerator Pedal Pos"/>
+        <filter val="Air Temp"/>
+        <filter val="Aux Rev Limiter Switch"/>
+        <filter val="Average Fuel Economy"/>
+        <filter val="Battery Light"/>
+        <filter val="Battery Voltage"/>
+        <filter val="Boost Control Output"/>
+        <filter val="Brake Pedal On"/>
+        <filter val="Brake Pressure"/>
+        <filter val="Clutch Switch"/>
+        <filter val="Coolant Pressure"/>
+        <filter val="Coolant Temp"/>
+        <filter val="Decel Cut"/>
+        <filter val="Diff Oil Temp"/>
+        <filter val="EGT 1"/>
+        <filter val="EGT 10"/>
+        <filter val="EGT 11"/>
+        <filter val="EGT 12"/>
+        <filter val="EGT 2"/>
+        <filter val="EGT 3"/>
+        <filter val="EGT 4"/>
+        <filter val="EGT 5"/>
+        <filter val="EGT 6"/>
+        <filter val="EGT 7"/>
+        <filter val="EGT 8"/>
+        <filter val="EGT 9"/>
+        <filter val="Exhaust Cam Angle #1"/>
+        <filter val="Exhaust Cam Angle #2"/>
+        <filter val="Flat Shift State"/>
+        <filter val="Fuel Composition"/>
+        <filter val="Fuel Composition Rate"/>
+        <filter val="Fuel Cut Percentage"/>
+        <filter val="Fuel Flow"/>
+        <filter val="Fuel Flow Differential"/>
+        <filter val="Fuel Flow Return"/>
+        <filter val="Fuel Pressure"/>
+        <filter val="Fuel Temp"/>
+        <filter val="Fuel Trim Long Term Bank 1"/>
+        <filter val="Fuel Trim Long Term Bank 2"/>
+        <filter val="Fuel Trim Short Term Bank 1"/>
+        <filter val="Fuel Trim Short Term Bank 2"/>
+        <filter val="Gear"/>
+        <filter val="Gear Switch State"/>
+        <filter val="Hand Brake Indicator"/>
+        <filter val="High Beam Indicator"/>
+        <filter val="Home Counter"/>
+        <filter val="Ignition Angle (Leading)"/>
+        <filter val="Ignition Angle (Trailing)"/>
+        <filter val="Injector Duty Cycle (Primary)"/>
+        <filter val="Intake Cam Angle #1"/>
+        <filter val="Knock Level Logged"/>
+        <filter val="Knock Level Logged 2"/>
+        <filter val="Knock Retard - Bank 1"/>
+        <filter val="Knock Retard - Bank 2"/>
+        <filter val="Lambda 1"/>
+        <filter val="Lambda 2"/>
+        <filter val="Lambda 3"/>
+        <filter val="Lambda 4"/>
+        <filter val="Launch Control Fuel Enrich"/>
+        <filter val="Launch Control Ign Retard"/>
+        <filter val="Left Indicator"/>
+        <filter val="Limp Mode Active"/>
+        <filter val="Manifold Pressure"/>
+        <filter val="Manifold Pressure 2"/>
+        <filter val="MIL (check engine light)"/>
+        <filter val="Miss Count"/>
+        <filter val="NOS Active"/>
+        <filter val="NOS Pressure"/>
+        <filter val="NOS Switch"/>
+        <filter val="Oil Pressure"/>
+        <filter val="Oil Temp"/>
+        <filter val="Rally Anti Lag Swich"/>
+        <filter val="Reserved (Distance to Empty)"/>
+        <filter val="Reserved (Fuel Level)"/>
+        <filter val="Right Indicator"/>
+        <filter val="RPM"/>
+        <filter val="Target Boost Level"/>
+        <filter val="Throttle Position"/>
+        <filter val="Timed Duty Output Active"/>
+        <filter val="Timed Duty Output Duty 1"/>
+        <filter val="Timed Duty Output Duty 2"/>
+        <filter val="Torque Reduction Active"/>
+        <filter val="Torque Reduction Cut Active"/>
+        <filter val="Transient Throttle Active"/>
+        <filter val="Transmission Oil Temp"/>
+        <filter val="Trigger Counter"/>
+        <filter val="Triggers Since Last Home"/>
+        <filter val="Turbo Speed Sensor"/>
+        <filter val="Wastegate Pressure"/>
+        <filter val="Wheel Diff"/>
+        <filter val="Wheel Slip"/>
+        <filter val="Wheelspeed Front"/>
+        <filter val="Wheelspeed Front Left"/>
+        <filter val="Wheelspeed Front Right"/>
+        <filter val="Wheelspeed General"/>
+        <filter val="Wheelspeed Rear"/>
+        <filter val="Wheelspeed Rear Left"/>
+        <filter val="Wheelspped Rear Right"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:M136"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -19633,7 +19089,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -19653,7 +19109,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B1:E639"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -27496,7 +26952,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G639"/>
+  <autoFilter ref="A1:G639" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>